<commit_message>
Build cleaned multi-source dashboard data
</commit_message>
<xml_diff>
--- a/data/merged/2026-08-31/MERGED_ES_Mite-Vacuum_2026-08-31.xlsx
+++ b/data/merged/2026-08-31/MERGED_ES_Mite-Vacuum_2026-08-31.xlsx
@@ -3703,13 +3703,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>192000</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>44999</xdr:rowOff>
+      <xdr:rowOff>45000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>428799</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>269999</xdr:rowOff>
+      <xdr:rowOff>270000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3835,13 +3835,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>192000</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>45000</xdr:rowOff>
+      <xdr:rowOff>44999</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>428799</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>270000</xdr:rowOff>
+      <xdr:rowOff>269999</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3946,50 +3946,6 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip r:embed="rId25" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>192000</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>44999</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>428799</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>269999</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="26" name="Product 26">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <ns2:creationId id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId26" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4331,7 +4287,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BR27"/>
+  <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -8512,45 +8468,45 @@
       <c r="B20" s="13"/>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>B0FBX24WH6</t>
+          <t>B0FDWVV95V</t>
         </is>
       </c>
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
       <c r="F20" s="14" t="inlineStr">
         <is>
-          <t>syayw</t>
+          <t>JIGOO</t>
         </is>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=syayw</t>
+          <t>https://www.amazon.es/stores/JIGOO-ES/page/23E9C8F3-B11D-41BE-B25B-391D7999E178?lp_asin=B0FDWVV95V&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto</t>
         </is>
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>syayw Limpiador Varuum – 68 W Fuerte Cama vacío para Limpieza ProfundasEliminador de para Mascotas vacío para Cojines de so</t>
+          <t>JIGOO T600 T600 - Tetina antiácaros/Floral Delight (aceite esencial de plantas)</t>
         </is>
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/dp/B0FBX24WH6?psc=1</t>
+          <t>https://www.amazon.es/dp/B0FDWVV95V?psc=1</t>
         </is>
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>https://images-na.ssl-images-amazon.com/images/I/61LvanTuKlL._AC_US600_.jpg</t>
+          <t>https://images-na.ssl-images-amazon.com/images/I/61tL+-AcL6L._AC_US600_.jpg</t>
         </is>
       </c>
       <c r="L20" s="14" t="inlineStr">
         <is>
-          <t>B0FBX24WH6</t>
+          <t>B0FDWVV95V</t>
         </is>
       </c>
       <c r="M20" s="14" t="inlineStr">
         <is>
-          <t>Hogar y cocina:Aspiración, limpieza y cuidado de suelo y ventanas:Aspiradoras:Aspiradoras de mano</t>
+          <t>Hogar y cocina:Aspiración, limpieza y cuidado de suelo y ventanas:Aspiradoras:Aspiradoras de futones</t>
         </is>
       </c>
       <c r="N20" s="14" t="inlineStr">
@@ -8559,22 +8515,22 @@
         </is>
       </c>
       <c r="O20" s="15">
-        <v>1528039</v>
-      </c>
-      <c r="P20" s="15"/>
+        <v>502605</v>
+      </c>
+      <c r="P20" s="15">
+        <v>-2214</v>
+      </c>
       <c r="Q20" s="16">
         <v>0</v>
       </c>
       <c r="R20" s="17" t="inlineStr">
         <is>
-          <t>Aspiradoras de futones
-Aspiradoras de mano</t>
+          <t>Aspiradoras de futones</t>
         </is>
       </c>
       <c r="S20" s="18" t="inlineStr">
         <is>
-          <t>25
-1817</t>
+          <t>14</t>
         </is>
       </c>
       <c r="T20" s="15"/>
@@ -8586,54 +8542,60 @@
         <v>1</v>
       </c>
       <c r="Z20" s="20">
-        <v>38.11</v>
+        <v>18.99</v>
       </c>
       <c r="AA20"/>
       <c r="AB20"/>
       <c r="AC20" s="2"/>
-      <c r="AD20" s="19"/>
-      <c r="AE20" s="15"/>
-      <c r="AF20" s="21"/>
+      <c r="AD20" s="19">
+        <v>10</v>
+      </c>
+      <c r="AE20" s="15">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="21">
+        <v>4.2</v>
+      </c>
       <c r="AG20" s="22">
         <v>0</v>
       </c>
       <c r="AH20" s="20">
-        <v>5.05</v>
+        <v>2.36</v>
       </c>
       <c r="AI20" s="16">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="AJ20"/>
       <c r="AK20" s="13" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="AL20" s="19">
-        <v>271</v>
+        <v>403</v>
       </c>
       <c r="AM20" s="13" t="inlineStr">
         <is>
-          <t>FBM</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AN20" s="13"/>
       <c r="AO20" s="13"/>
       <c r="AP20"/>
       <c r="AQ20" s="19">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AR20" s="19">
         <v>1</v>
       </c>
       <c r="AS20" s="14" t="inlineStr">
         <is>
-          <t>nousaeg</t>
+          <t>tengjidainzi</t>
         </is>
       </c>
       <c r="AT20" s="13" t="inlineStr">
         <is>
-          <t>FBM</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AU20" s="13" t="inlineStr">
@@ -8643,12 +8605,12 @@
       </c>
       <c r="AV20" s="14" t="inlineStr">
         <is>
-          <t>蚌埠市 蚌山区 安徽 233000 CN</t>
+          <t>深圳市 广东 518033 CN</t>
         </is>
       </c>
       <c r="AW20" s="13" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A3T9BSXCSWI46M</t>
+          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A1LBASE3VLPMEX</t>
         </is>
       </c>
       <c r="AX20" s="13"/>
@@ -8656,11 +8618,7 @@
       <c r="AZ20" s="13"/>
       <c r="BA20" s="13"/>
       <c r="BB20" s="13"/>
-      <c r="BC20" s="13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="BC20" s="13"/>
       <c r="BD20" s="13"/>
       <c r="BE20" s="13"/>
       <c r="BF20" s="13"/>
@@ -8669,47 +8627,43 @@
       <c r="BI20" s="23"/>
       <c r="BJ20" s="23" t="inlineStr">
         <is>
-          <t>1,02 kg</t>
+          <t>50 g</t>
         </is>
       </c>
       <c r="BK20" s="23" t="inlineStr">
         <is>
-          <t>1.02 kg</t>
+          <t>50.00 g</t>
         </is>
       </c>
       <c r="BL20" s="23" t="inlineStr">
         <is>
-          <t>26.9 x 25.2 x 14.3 cm</t>
-        </is>
-      </c>
-      <c r="BM20" s="23" t="inlineStr">
-        <is>
-          <t>26.90 x 25.20 x 14.30 cm</t>
-        </is>
-      </c>
+          <t>6l. x 1,3an. x 8al. centímetros</t>
+        </is>
+      </c>
+      <c r="BM20" s="23"/>
       <c r="BN20" s="23" t="inlineStr">
         <is>
-          <t>1.02 kg</t>
+          <t>50 g</t>
         </is>
       </c>
       <c r="BO20" s="23" t="inlineStr">
         <is>
-          <t>1.02 kg</t>
+          <t>50.00 g</t>
         </is>
       </c>
       <c r="BP20" s="23" t="inlineStr">
         <is>
-          <t>26.9 x 25.2 x 14.3 cm</t>
+          <t>10 x 6 x 1.5 cm</t>
         </is>
       </c>
       <c r="BQ20" s="23" t="inlineStr">
         <is>
-          <t>26.90 x 25.20 x 14.30 cm</t>
+          <t>10.00 x 6.00 x 1.50 cm</t>
         </is>
       </c>
       <c r="BR20" s="13" t="inlineStr">
         <is>
-          <t>标准包裹</t>
+          <t>轻型信封</t>
         </is>
       </c>
     </row>
@@ -8720,40 +8674,40 @@
       <c r="B21" s="13"/>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>B0FDWVV95V</t>
+          <t>B0FKRC3KQY</t>
         </is>
       </c>
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>JIGOO</t>
+          <t>Yaasier</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/stores/JIGOO-ES/page/23E9C8F3-B11D-41BE-B25B-391D7999E178?lp_asin=B0FDWVV95V&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto</t>
+          <t>https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Yaasier</t>
         </is>
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>JIGOO T600 T600 - Tetina antiácaros/Floral Delight (aceite esencial de plantas)</t>
+          <t>Yaasier Aspirador de Ácaros, Mini Aspirador Antiácaros para Colchones con Luz UV, Aspiradora de Mano con Filtro HEPA para Col</t>
         </is>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/dp/B0FDWVV95V?psc=1</t>
+          <t>https://www.amazon.es/dp/B0FKRC3KQY?psc=1</t>
         </is>
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>https://images-na.ssl-images-amazon.com/images/I/61tL+-AcL6L._AC_US600_.jpg</t>
+          <t>https://images-na.ssl-images-amazon.com/images/I/511XZVAimmL._AC_US600_.jpg</t>
         </is>
       </c>
       <c r="L21" s="14" t="inlineStr">
         <is>
-          <t>B0FDWVV95V</t>
+          <t>B0FKRC3KQY</t>
         </is>
       </c>
       <c r="M21" s="14" t="inlineStr">
@@ -8767,11 +8721,9 @@
         </is>
       </c>
       <c r="O21" s="15">
-        <v>502605</v>
-      </c>
-      <c r="P21" s="15">
-        <v>-2214</v>
-      </c>
+        <v>464021</v>
+      </c>
+      <c r="P21" s="15"/>
       <c r="Q21" s="16">
         <v>0</v>
       </c>
@@ -8782,7 +8734,7 @@
       </c>
       <c r="S21" s="18" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="T21" s="15"/>
@@ -8794,37 +8746,37 @@
         <v>1</v>
       </c>
       <c r="Z21" s="20">
-        <v>18.99</v>
+        <v>25.99</v>
       </c>
       <c r="AA21"/>
       <c r="AB21"/>
       <c r="AC21" s="2"/>
       <c r="AD21" s="19">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AE21" s="15">
         <v>0</v>
       </c>
       <c r="AF21" s="21">
-        <v>4.2</v>
+        <v>3.3</v>
       </c>
       <c r="AG21" s="22">
         <v>0</v>
       </c>
       <c r="AH21" s="20">
-        <v>2.36</v>
+        <v>4.11</v>
       </c>
       <c r="AI21" s="16">
-        <v>0.73</v>
+        <v>0.69</v>
       </c>
       <c r="AJ21"/>
       <c r="AK21" s="13" t="inlineStr">
         <is>
-          <t>2025-07-23</t>
+          <t>2025-08-31</t>
         </is>
       </c>
       <c r="AL21" s="19">
-        <v>403</v>
+        <v>365</v>
       </c>
       <c r="AM21" s="13" t="inlineStr">
         <is>
@@ -8835,14 +8787,14 @@
       <c r="AO21" s="13"/>
       <c r="AP21"/>
       <c r="AQ21" s="19">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="AR21" s="19">
         <v>1</v>
       </c>
       <c r="AS21" s="14" t="inlineStr">
         <is>
-          <t>tengjidainzi</t>
+          <t>Renyu</t>
         </is>
       </c>
       <c r="AT21" s="13" t="inlineStr">
@@ -8857,12 +8809,12 @@
       </c>
       <c r="AV21" s="14" t="inlineStr">
         <is>
-          <t>深圳市 广东 518033 CN</t>
+          <t>dong hu xin ji shu hubei 430223 CN</t>
         </is>
       </c>
       <c r="AW21" s="13" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A1LBASE3VLPMEX</t>
+          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=ATK258MBI08TX</t>
         </is>
       </c>
       <c r="AX21" s="13"/>
@@ -8870,7 +8822,11 @@
       <c r="AZ21" s="13"/>
       <c r="BA21" s="13"/>
       <c r="BB21" s="13"/>
-      <c r="BC21" s="13"/>
+      <c r="BC21" s="13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="BD21" s="13"/>
       <c r="BE21" s="13"/>
       <c r="BF21" s="13"/>
@@ -8879,43 +8835,47 @@
       <c r="BI21" s="23"/>
       <c r="BJ21" s="23" t="inlineStr">
         <is>
-          <t>50 g</t>
+          <t>400 g</t>
         </is>
       </c>
       <c r="BK21" s="23" t="inlineStr">
         <is>
-          <t>50.00 g</t>
+          <t>400.00 g</t>
         </is>
       </c>
       <c r="BL21" s="23" t="inlineStr">
         <is>
-          <t>6l. x 1,3an. x 8al. centímetros</t>
-        </is>
-      </c>
-      <c r="BM21" s="23"/>
+          <t>4 x 4 x 8 cm</t>
+        </is>
+      </c>
+      <c r="BM21" s="23" t="inlineStr">
+        <is>
+          <t>4.00 x 4.00 x 8.00 cm</t>
+        </is>
+      </c>
       <c r="BN21" s="23" t="inlineStr">
         <is>
-          <t>50 g</t>
+          <t>400 g</t>
         </is>
       </c>
       <c r="BO21" s="23" t="inlineStr">
         <is>
-          <t>50.00 g</t>
+          <t>400.00 g</t>
         </is>
       </c>
       <c r="BP21" s="23" t="inlineStr">
         <is>
-          <t>10 x 6 x 1.5 cm</t>
+          <t>23.2 x 11.7 x 10.2 cm</t>
         </is>
       </c>
       <c r="BQ21" s="23" t="inlineStr">
         <is>
-          <t>10.00 x 6.00 x 1.50 cm</t>
+          <t>23.20 x 11.70 x 10.20 cm</t>
         </is>
       </c>
       <c r="BR21" s="13" t="inlineStr">
         <is>
-          <t>轻型信封</t>
+          <t>小包裹</t>
         </is>
       </c>
     </row>
@@ -8926,40 +8886,40 @@
       <c r="B22" s="13"/>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>B0FKRC3KQY</t>
+          <t>B0FN3GPQZM</t>
         </is>
       </c>
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>Yaasier</t>
+          <t>Teant</t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Yaasier</t>
+          <t>https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Teant</t>
         </is>
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>Yaasier Aspirador de Ácaros, Mini Aspirador Antiácaros para Colchones con Luz UV, Aspiradora de Mano con Filtro HEPA para Col</t>
+          <t>Mayking Teant Aspiradora para Colchones 2 Velocidades (14 kPa/18 kPa)</t>
         </is>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/dp/B0FKRC3KQY?psc=1</t>
+          <t>https://www.amazon.es/dp/B0FN3GPQZM?psc=1</t>
         </is>
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>https://images-na.ssl-images-amazon.com/images/I/511XZVAimmL._AC_US600_.jpg</t>
+          <t>https://images-na.ssl-images-amazon.com/images/I/71gt+j80L3L._AC_US600_.jpg</t>
         </is>
       </c>
       <c r="L22" s="14" t="inlineStr">
         <is>
-          <t>B0FKRC3KQY</t>
+          <t>B0FN3GPQZM</t>
         </is>
       </c>
       <c r="M22" s="14" t="inlineStr">
@@ -8973,7 +8933,7 @@
         </is>
       </c>
       <c r="O22" s="15">
-        <v>464021</v>
+        <v>331819</v>
       </c>
       <c r="P22" s="15"/>
       <c r="Q22" s="16">
@@ -8986,7 +8946,7 @@
       </c>
       <c r="S22" s="18" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="T22" s="15"/>
@@ -8998,41 +8958,41 @@
         <v>1</v>
       </c>
       <c r="Z22" s="20">
-        <v>25.99</v>
+        <v>126.51</v>
       </c>
       <c r="AA22"/>
       <c r="AB22"/>
       <c r="AC22" s="2"/>
       <c r="AD22" s="19">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="AE22" s="15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AF22" s="21">
-        <v>3.3</v>
+        <v>4.6</v>
       </c>
       <c r="AG22" s="22">
         <v>0</v>
       </c>
       <c r="AH22" s="20">
-        <v>4.11</v>
+        <v>8.37</v>
       </c>
       <c r="AI22" s="16">
-        <v>0.69</v>
+        <v>0.78</v>
       </c>
       <c r="AJ22"/>
       <c r="AK22" s="13" t="inlineStr">
         <is>
-          <t>2025-08-31</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="AL22" s="19">
-        <v>365</v>
+        <v>248</v>
       </c>
       <c r="AM22" s="13" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>FBA</t>
         </is>
       </c>
       <c r="AN22" s="13"/>
@@ -9046,12 +9006,12 @@
       </c>
       <c r="AS22" s="14" t="inlineStr">
         <is>
-          <t>Renyu</t>
+          <t>Teant</t>
         </is>
       </c>
       <c r="AT22" s="13" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>FBA</t>
         </is>
       </c>
       <c r="AU22" s="13" t="inlineStr">
@@ -9061,12 +9021,12 @@
       </c>
       <c r="AV22" s="14" t="inlineStr">
         <is>
-          <t>dong hu xin ji shu hubei 430223 CN</t>
+          <t>郑州市 河南 450000 CN</t>
         </is>
       </c>
       <c r="AW22" s="13" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=ATK258MBI08TX</t>
+          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A3EVTWEH1TBVG5</t>
         </is>
       </c>
       <c r="AX22" s="13"/>
@@ -9087,47 +9047,47 @@
       <c r="BI22" s="23"/>
       <c r="BJ22" s="23" t="inlineStr">
         <is>
-          <t>400 g</t>
+          <t>1.9 kg</t>
         </is>
       </c>
       <c r="BK22" s="23" t="inlineStr">
         <is>
-          <t>400.00 g</t>
+          <t>1.90 kg</t>
         </is>
       </c>
       <c r="BL22" s="23" t="inlineStr">
         <is>
-          <t>4 x 4 x 8 cm</t>
+          <t>36 x 29 x 25 cm</t>
         </is>
       </c>
       <c r="BM22" s="23" t="inlineStr">
         <is>
-          <t>4.00 x 4.00 x 8.00 cm</t>
+          <t>36.00 x 29.00 x 25.00 cm</t>
         </is>
       </c>
       <c r="BN22" s="23" t="inlineStr">
         <is>
-          <t>400 g</t>
+          <t>2.6 kg</t>
         </is>
       </c>
       <c r="BO22" s="23" t="inlineStr">
         <is>
-          <t>400.00 g</t>
+          <t>2.60 kg</t>
         </is>
       </c>
       <c r="BP22" s="23" t="inlineStr">
         <is>
-          <t>23.2 x 11.7 x 10.2 cm</t>
+          <t>33.3 x 28.1 x 27.2 cm</t>
         </is>
       </c>
       <c r="BQ22" s="23" t="inlineStr">
         <is>
-          <t>23.20 x 11.70 x 10.20 cm</t>
+          <t>33.30 x 28.10 x 27.20 cm</t>
         </is>
       </c>
       <c r="BR22" s="13" t="inlineStr">
         <is>
-          <t>小包裹</t>
+          <t>轻型标准大件</t>
         </is>
       </c>
     </row>
@@ -9138,40 +9098,40 @@
       <c r="B23" s="13"/>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>B0FN3GPQZM</t>
+          <t>B0FVS559GZ</t>
         </is>
       </c>
       <c r="D23" s="14"/>
       <c r="E23" s="14"/>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Teant</t>
+          <t>Yaasier</t>
         </is>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Teant</t>
+          <t>https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Yaasier</t>
         </is>
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>Mayking Teant Aspiradora para Colchones 2 Velocidades (14 kPa/18 kPa)</t>
+          <t>Yaasier Aspirador de ácaros con luz UV, Mini aspiradora con Filtro HEPA, Aspirador antiacaros con depósito de Polvo Permanent</t>
         </is>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/dp/B0FN3GPQZM?psc=1</t>
+          <t>https://www.amazon.es/dp/B0FVS559GZ?psc=1</t>
         </is>
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>https://images-na.ssl-images-amazon.com/images/I/71gt+j80L3L._AC_US600_.jpg</t>
+          <t>https://images-na.ssl-images-amazon.com/images/I/51dJLeDXofL._AC_US600_.jpg</t>
         </is>
       </c>
       <c r="L23" s="14" t="inlineStr">
         <is>
-          <t>B0FN3GPQZM</t>
+          <t>B0FVS559GZ</t>
         </is>
       </c>
       <c r="M23" s="14" t="inlineStr">
@@ -9185,7 +9145,7 @@
         </is>
       </c>
       <c r="O23" s="15">
-        <v>331819</v>
+        <v>308552</v>
       </c>
       <c r="P23" s="15"/>
       <c r="Q23" s="16">
@@ -9198,7 +9158,7 @@
       </c>
       <c r="S23" s="18" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="T23" s="15"/>
@@ -9210,41 +9170,41 @@
         <v>1</v>
       </c>
       <c r="Z23" s="20">
-        <v>126.51</v>
+        <v>23.99</v>
       </c>
       <c r="AA23"/>
       <c r="AB23"/>
       <c r="AC23" s="2"/>
       <c r="AD23" s="19">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="AE23" s="15">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF23" s="21">
-        <v>4.6</v>
+        <v>3.6</v>
       </c>
       <c r="AG23" s="22">
         <v>0</v>
       </c>
       <c r="AH23" s="20">
-        <v>8.37</v>
+        <v>4.11</v>
       </c>
       <c r="AI23" s="16">
-        <v>0.78</v>
+        <v>0.68</v>
       </c>
       <c r="AJ23"/>
       <c r="AK23" s="13" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-10-20</t>
         </is>
       </c>
       <c r="AL23" s="19">
-        <v>248</v>
+        <v>314</v>
       </c>
       <c r="AM23" s="13" t="inlineStr">
         <is>
-          <t>FBA</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AN23" s="13"/>
@@ -9258,12 +9218,12 @@
       </c>
       <c r="AS23" s="14" t="inlineStr">
         <is>
-          <t>Teant</t>
+          <t>Renyu</t>
         </is>
       </c>
       <c r="AT23" s="13" t="inlineStr">
         <is>
-          <t>FBA</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AU23" s="13" t="inlineStr">
@@ -9273,12 +9233,12 @@
       </c>
       <c r="AV23" s="14" t="inlineStr">
         <is>
-          <t>郑州市 河南 450000 CN</t>
+          <t>dong hu xin ji shu hubei 430223 CN</t>
         </is>
       </c>
       <c r="AW23" s="13" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A3EVTWEH1TBVG5</t>
+          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=ATK258MBI08TX</t>
         </is>
       </c>
       <c r="AX23" s="13"/>
@@ -9291,7 +9251,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="BD23" s="13"/>
+      <c r="BD23" s="13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="BE23" s="13"/>
       <c r="BF23" s="13"/>
       <c r="BG23" s="13"/>
@@ -9299,47 +9263,47 @@
       <c r="BI23" s="23"/>
       <c r="BJ23" s="23" t="inlineStr">
         <is>
-          <t>1.9 kg</t>
+          <t>250 g</t>
         </is>
       </c>
       <c r="BK23" s="23" t="inlineStr">
         <is>
-          <t>1.90 kg</t>
+          <t>250.00 g</t>
         </is>
       </c>
       <c r="BL23" s="23" t="inlineStr">
         <is>
-          <t>36 x 29 x 25 cm</t>
+          <t>6 x 4 x 8 cm</t>
         </is>
       </c>
       <c r="BM23" s="23" t="inlineStr">
         <is>
-          <t>36.00 x 29.00 x 25.00 cm</t>
+          <t>6.00 x 4.00 x 8.00 cm</t>
         </is>
       </c>
       <c r="BN23" s="23" t="inlineStr">
         <is>
-          <t>2.6 kg</t>
+          <t>400 g</t>
         </is>
       </c>
       <c r="BO23" s="23" t="inlineStr">
         <is>
-          <t>2.60 kg</t>
+          <t>400.00 g</t>
         </is>
       </c>
       <c r="BP23" s="23" t="inlineStr">
         <is>
-          <t>33.3 x 28.1 x 27.2 cm</t>
+          <t>23.1 x 11.7 x 10.2 cm</t>
         </is>
       </c>
       <c r="BQ23" s="23" t="inlineStr">
         <is>
-          <t>33.30 x 28.10 x 27.20 cm</t>
+          <t>23.10 x 11.70 x 10.20 cm</t>
         </is>
       </c>
       <c r="BR23" s="13" t="inlineStr">
         <is>
-          <t>轻型标准大件</t>
+          <t>小包裹</t>
         </is>
       </c>
     </row>
@@ -9350,7 +9314,7 @@
       <c r="B24" s="13"/>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>B0FVS559GZ</t>
+          <t>B0FYM1D13D</t>
         </is>
       </c>
       <c r="D24" s="14"/>
@@ -9367,13 +9331,13 @@
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>Yaasier Aspirador de ácaros con luz UV, Mini aspiradora con Filtro HEPA, Aspirador antiacaros con depósito de Polvo Permanent</t>
+          <t>Aspirador de ácaros con luz UV, Mini aspiradora con Filtro HEPA, Aspirador antiacaros con depósito de Polvo Permanente para c</t>
         </is>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/dp/B0FVS559GZ?psc=1</t>
+          <t>https://www.amazon.es/dp/B0FYM1D13D?psc=1</t>
         </is>
       </c>
       <c r="K24" s="14" t="inlineStr">
@@ -9383,7 +9347,7 @@
       </c>
       <c r="L24" s="14" t="inlineStr">
         <is>
-          <t>B0FVS559GZ</t>
+          <t>B0FYM1D13D</t>
         </is>
       </c>
       <c r="M24" s="14" t="inlineStr">
@@ -9397,7 +9361,7 @@
         </is>
       </c>
       <c r="O24" s="15">
-        <v>308552</v>
+        <v>1135692</v>
       </c>
       <c r="P24" s="15"/>
       <c r="Q24" s="16">
@@ -9410,7 +9374,7 @@
       </c>
       <c r="S24" s="18" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>22</t>
         </is>
       </c>
       <c r="T24" s="15"/>
@@ -9422,19 +9386,19 @@
         <v>1</v>
       </c>
       <c r="Z24" s="20">
-        <v>23.99</v>
+        <v>26.99</v>
       </c>
       <c r="AA24"/>
       <c r="AB24"/>
       <c r="AC24" s="2"/>
       <c r="AD24" s="19">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="AE24" s="15">
         <v>0</v>
       </c>
       <c r="AF24" s="21">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="AG24" s="22">
         <v>0</v>
@@ -9443,16 +9407,16 @@
         <v>4.11</v>
       </c>
       <c r="AI24" s="16">
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
       <c r="AJ24"/>
       <c r="AK24" s="13" t="inlineStr">
         <is>
-          <t>2025-10-20</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="AL24" s="19">
-        <v>314</v>
+        <v>279</v>
       </c>
       <c r="AM24" s="13" t="inlineStr">
         <is>
@@ -9463,7 +9427,7 @@
       <c r="AO24" s="13"/>
       <c r="AP24"/>
       <c r="AQ24" s="19">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AR24" s="19">
         <v>1</v>
@@ -9503,11 +9467,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="BD24" s="13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="BD24" s="13"/>
       <c r="BE24" s="13"/>
       <c r="BF24" s="13"/>
       <c r="BG24" s="13"/>
@@ -9515,24 +9475,20 @@
       <c r="BI24" s="23"/>
       <c r="BJ24" s="23" t="inlineStr">
         <is>
-          <t>250 g</t>
+          <t>400 g</t>
         </is>
       </c>
       <c r="BK24" s="23" t="inlineStr">
         <is>
-          <t>250.00 g</t>
+          <t>400.00 g</t>
         </is>
       </c>
       <c r="BL24" s="23" t="inlineStr">
         <is>
-          <t>6 x 4 x 8 cm</t>
-        </is>
-      </c>
-      <c r="BM24" s="23" t="inlineStr">
-        <is>
-          <t>6.00 x 4.00 x 8.00 cm</t>
-        </is>
-      </c>
+          <t>6l. x 4an. x 8al. centímetros</t>
+        </is>
+      </c>
+      <c r="BM24" s="23"/>
       <c r="BN24" s="23" t="inlineStr">
         <is>
           <t>400 g</t>
@@ -9545,12 +9501,12 @@
       </c>
       <c r="BP24" s="23" t="inlineStr">
         <is>
-          <t>23.1 x 11.7 x 10.2 cm</t>
+          <t>23.8 x 11.7 x 10.2 cm</t>
         </is>
       </c>
       <c r="BQ24" s="23" t="inlineStr">
         <is>
-          <t>23.10 x 11.70 x 10.20 cm</t>
+          <t>23.80 x 11.70 x 10.20 cm</t>
         </is>
       </c>
       <c r="BR24" s="13" t="inlineStr">
@@ -9566,40 +9522,40 @@
       <c r="B25" s="13"/>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>B0FYM1D13D</t>
+          <t>B0G4RSJQVT</t>
         </is>
       </c>
       <c r="D25" s="14"/>
       <c r="E25" s="14"/>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>Yaasier</t>
+          <t>Lubluelu</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Yaasier</t>
+          <t>https://www.amazon.es/stores/Lubluelu/page/6949B717-1950-436B-B468-8BFB57AEF209?lp_asin=B0G4RSJQVT&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto&amp;bl_grd_status=override</t>
         </is>
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>Aspirador de ácaros con luz UV, Mini aspiradora con Filtro HEPA, Aspirador antiacaros con depósito de Polvo Permanente para c</t>
+          <t>Lubluelu Aspirador de ácaros 3 en 1 para colchones, 18 KPa fuerte potencia de succión, limpiador de colchones contra ácaros,</t>
         </is>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/dp/B0FYM1D13D?psc=1</t>
+          <t>https://www.amazon.es/dp/B0G4RSJQVT?psc=1</t>
         </is>
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>https://images-na.ssl-images-amazon.com/images/I/51dJLeDXofL._AC_US600_.jpg</t>
+          <t>https://images-na.ssl-images-amazon.com/images/I/71mJa10XC6L._AC_US600_.jpg</t>
         </is>
       </c>
       <c r="L25" s="14" t="inlineStr">
         <is>
-          <t>B0FYM1D13D</t>
+          <t>B0G4RSJQVT</t>
         </is>
       </c>
       <c r="M25" s="14" t="inlineStr">
@@ -9613,11 +9569,13 @@
         </is>
       </c>
       <c r="O25" s="15">
-        <v>1135692</v>
-      </c>
-      <c r="P25" s="15"/>
+        <v>1011527</v>
+      </c>
+      <c r="P25" s="15">
+        <v>-9945</v>
+      </c>
       <c r="Q25" s="16">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="R25" s="17" t="inlineStr">
         <is>
@@ -9626,7 +9584,7 @@
       </c>
       <c r="S25" s="18" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>19</t>
         </is>
       </c>
       <c r="T25" s="15"/>
@@ -9638,37 +9596,37 @@
         <v>1</v>
       </c>
       <c r="Z25" s="20">
-        <v>26.99</v>
+        <v>71.58</v>
       </c>
       <c r="AA25"/>
       <c r="AB25"/>
       <c r="AC25" s="2"/>
       <c r="AD25" s="19">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="AE25" s="15">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="AF25" s="21">
-        <v>3</v>
+        <v>4.6</v>
       </c>
       <c r="AG25" s="22">
         <v>0</v>
       </c>
       <c r="AH25" s="20">
-        <v>4.11</v>
+        <v>5.8</v>
       </c>
       <c r="AI25" s="16">
-        <v>0.7</v>
+        <v>0.77</v>
       </c>
       <c r="AJ25"/>
       <c r="AK25" s="13" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="AL25" s="19">
-        <v>279</v>
+        <v>173</v>
       </c>
       <c r="AM25" s="13" t="inlineStr">
         <is>
@@ -9686,7 +9644,7 @@
       </c>
       <c r="AS25" s="14" t="inlineStr">
         <is>
-          <t>Renyu</t>
+          <t>Amazon Segunda mano</t>
         </is>
       </c>
       <c r="AT25" s="13" t="inlineStr">
@@ -9694,31 +9652,15 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="AU25" s="13" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="AV25" s="14" t="inlineStr">
-        <is>
-          <t>dong hu xin ji shu hubei 430223 CN</t>
-        </is>
-      </c>
-      <c r="AW25" s="13" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=ATK258MBI08TX</t>
-        </is>
-      </c>
+      <c r="AU25" s="13"/>
+      <c r="AV25" s="14"/>
+      <c r="AW25" s="13"/>
       <c r="AX25" s="13"/>
       <c r="AY25" s="13"/>
       <c r="AZ25" s="13"/>
       <c r="BA25" s="13"/>
       <c r="BB25" s="13"/>
-      <c r="BC25" s="13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="BC25" s="13"/>
       <c r="BD25" s="13"/>
       <c r="BE25" s="13"/>
       <c r="BF25" s="13"/>
@@ -9727,43 +9669,47 @@
       <c r="BI25" s="23"/>
       <c r="BJ25" s="23" t="inlineStr">
         <is>
-          <t>400 g</t>
+          <t>2,33 kg</t>
         </is>
       </c>
       <c r="BK25" s="23" t="inlineStr">
         <is>
-          <t>400.00 g</t>
+          <t>2.33 kg</t>
         </is>
       </c>
       <c r="BL25" s="23" t="inlineStr">
         <is>
-          <t>6l. x 4an. x 8al. centímetros</t>
-        </is>
-      </c>
-      <c r="BM25" s="23"/>
+          <t>42 x 31 x 18 cm</t>
+        </is>
+      </c>
+      <c r="BM25" s="23" t="inlineStr">
+        <is>
+          <t>42.00 x 31.00 x 18.00 cm</t>
+        </is>
+      </c>
       <c r="BN25" s="23" t="inlineStr">
         <is>
-          <t>400 g</t>
+          <t>2.33 kg</t>
         </is>
       </c>
       <c r="BO25" s="23" t="inlineStr">
         <is>
-          <t>400.00 g</t>
+          <t>2.33 kg</t>
         </is>
       </c>
       <c r="BP25" s="23" t="inlineStr">
         <is>
-          <t>23.8 x 11.7 x 10.2 cm</t>
+          <t>33.6 x 26.9 x 25.6 cm</t>
         </is>
       </c>
       <c r="BQ25" s="23" t="inlineStr">
         <is>
-          <t>23.80 x 11.70 x 10.20 cm</t>
+          <t>33.60 x 26.90 x 25.60 cm</t>
         </is>
       </c>
       <c r="BR25" s="13" t="inlineStr">
         <is>
-          <t>小包裹</t>
+          <t>标准包裹</t>
         </is>
       </c>
     </row>
@@ -9774,40 +9720,40 @@
       <c r="B26" s="13"/>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>B0G4RSJQVT</t>
+          <t>B0GYS43G8G</t>
         </is>
       </c>
       <c r="D26" s="14"/>
       <c r="E26" s="14"/>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>Lubluelu</t>
+          <t>ALLILUYAA</t>
         </is>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/stores/Lubluelu/page/6949B717-1950-436B-B468-8BFB57AEF209?lp_asin=B0G4RSJQVT&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto&amp;bl_grd_status=override</t>
+          <t>https://www.amazon.es/stores/ALILILUYAA/page/6F2D9C3F-3247-41D0-93BE-BD3270082609?lp_asin=B0GYS43G8G&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto&amp;bl_grd_status=override</t>
         </is>
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>Lubluelu Aspirador de ácaros 3 en 1 para colchones, 18 KPa fuerte potencia de succión, limpiador de colchones contra ácaros,</t>
+          <t>Aspiradora De Acaros, Aspiradora Antiacaros con Triple Filtración Y Filtro Lavable, Vibración De Alta Frecuencia, Maquina Ant</t>
         </is>
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/dp/B0G4RSJQVT?psc=1</t>
+          <t>https://www.amazon.es/dp/B0GYS43G8G?psc=1</t>
         </is>
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>https://images-na.ssl-images-amazon.com/images/I/71mJa10XC6L._AC_US600_.jpg</t>
+          <t>https://images-na.ssl-images-amazon.com/images/I/51JXrvAAoZL._AC_US600_.jpg</t>
         </is>
       </c>
       <c r="L26" s="14" t="inlineStr">
         <is>
-          <t>B0G4RSJQVT</t>
+          <t>B0GYS43G8G</t>
         </is>
       </c>
       <c r="M26" s="14" t="inlineStr">
@@ -9821,13 +9767,13 @@
         </is>
       </c>
       <c r="O26" s="15">
-        <v>1011527</v>
+        <v>588206</v>
       </c>
       <c r="P26" s="15">
-        <v>-9945</v>
+        <v>-26517</v>
       </c>
       <c r="Q26" s="16">
-        <v>-0.01</v>
+        <v>-0.05</v>
       </c>
       <c r="R26" s="17" t="inlineStr">
         <is>
@@ -9836,7 +9782,7 @@
       </c>
       <c r="S26" s="18" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>16</t>
         </is>
       </c>
       <c r="T26" s="15"/>
@@ -9848,37 +9794,37 @@
         <v>1</v>
       </c>
       <c r="Z26" s="20">
-        <v>71.58</v>
+        <v>25.99</v>
       </c>
       <c r="AA26"/>
       <c r="AB26"/>
       <c r="AC26" s="2"/>
       <c r="AD26" s="19">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="AE26" s="15">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="AF26" s="21">
-        <v>4.6</v>
+        <v>1</v>
       </c>
       <c r="AG26" s="22">
         <v>0</v>
       </c>
       <c r="AH26" s="20">
-        <v>5.8</v>
+        <v>4.37</v>
       </c>
       <c r="AI26" s="16">
-        <v>0.77</v>
+        <v>0.68</v>
       </c>
       <c r="AJ26"/>
       <c r="AK26" s="13" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="AL26" s="19">
-        <v>173</v>
+        <v>88</v>
       </c>
       <c r="AM26" s="13" t="inlineStr">
         <is>
@@ -9889,14 +9835,14 @@
       <c r="AO26" s="13"/>
       <c r="AP26"/>
       <c r="AQ26" s="19">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AR26" s="19">
         <v>1</v>
       </c>
       <c r="AS26" s="14" t="inlineStr">
         <is>
-          <t>Amazon Segunda mano</t>
+          <t>ALLILUYAA</t>
         </is>
       </c>
       <c r="AT26" s="13" t="inlineStr">
@@ -9904,9 +9850,21 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="AU26" s="13"/>
-      <c r="AV26" s="14"/>
-      <c r="AW26" s="13"/>
+      <c r="AU26" s="13" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="AV26" s="14" t="inlineStr">
+        <is>
+          <t>bayuquan LiaoNing 115007 CN</t>
+        </is>
+      </c>
+      <c r="AW26" s="13" t="inlineStr">
+        <is>
+          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A238ODZG8O3E58</t>
+        </is>
+      </c>
       <c r="AX26" s="13"/>
       <c r="AY26" s="13"/>
       <c r="AZ26" s="13"/>
@@ -9919,249 +9877,39 @@
       <c r="BG26" s="13"/>
       <c r="BH26" s="14"/>
       <c r="BI26" s="23"/>
-      <c r="BJ26" s="23" t="inlineStr">
-        <is>
-          <t>2,33 kg</t>
-        </is>
-      </c>
-      <c r="BK26" s="23" t="inlineStr">
-        <is>
-          <t>2.33 kg</t>
-        </is>
-      </c>
+      <c r="BJ26" s="23"/>
+      <c r="BK26" s="23"/>
       <c r="BL26" s="23" t="inlineStr">
         <is>
-          <t>42 x 31 x 18 cm</t>
+          <t>1 x 1 x 1 cm</t>
         </is>
       </c>
       <c r="BM26" s="23" t="inlineStr">
         <is>
-          <t>42.00 x 31.00 x 18.00 cm</t>
+          <t>1.00 x 1.00 x 1.00 cm</t>
         </is>
       </c>
       <c r="BN26" s="23" t="inlineStr">
         <is>
-          <t>2.33 kg</t>
+          <t>430 g</t>
         </is>
       </c>
       <c r="BO26" s="23" t="inlineStr">
         <is>
-          <t>2.33 kg</t>
+          <t>430.00 g</t>
         </is>
       </c>
       <c r="BP26" s="23" t="inlineStr">
         <is>
-          <t>33.6 x 26.9 x 25.6 cm</t>
+          <t>25.1 x 20.5 x 11.2 cm</t>
         </is>
       </c>
       <c r="BQ26" s="23" t="inlineStr">
         <is>
-          <t>33.60 x 26.90 x 25.60 cm</t>
+          <t>25.10 x 20.50 x 11.20 cm</t>
         </is>
       </c>
       <c r="BR26" s="13" t="inlineStr">
-        <is>
-          <t>标准包裹</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="13">
-        <v>26</v>
-      </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>B0GYS43G8G</t>
-        </is>
-      </c>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>ALLILUYAA</t>
-        </is>
-      </c>
-      <c r="G27" s="14" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/stores/ALILILUYAA/page/6F2D9C3F-3247-41D0-93BE-BD3270082609?lp_asin=B0GYS43G8G&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto&amp;bl_grd_status=override</t>
-        </is>
-      </c>
-      <c r="H27" s="14" t="inlineStr">
-        <is>
-          <t>Aspiradora De Acaros, Aspiradora Antiacaros con Triple Filtración Y Filtro Lavable, Vibración De Alta Frecuencia, Maquina Ant</t>
-        </is>
-      </c>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/dp/B0GYS43G8G?psc=1</t>
-        </is>
-      </c>
-      <c r="K27" s="14" t="inlineStr">
-        <is>
-          <t>https://images-na.ssl-images-amazon.com/images/I/51JXrvAAoZL._AC_US600_.jpg</t>
-        </is>
-      </c>
-      <c r="L27" s="14" t="inlineStr">
-        <is>
-          <t>B0GYS43G8G</t>
-        </is>
-      </c>
-      <c r="M27" s="14" t="inlineStr">
-        <is>
-          <t>Hogar y cocina:Aspiración, limpieza y cuidado de suelo y ventanas:Aspiradoras:Aspiradoras de futones</t>
-        </is>
-      </c>
-      <c r="N27" s="14" t="inlineStr">
-        <is>
-          <t>Hogar y cocina</t>
-        </is>
-      </c>
-      <c r="O27" s="15">
-        <v>588206</v>
-      </c>
-      <c r="P27" s="15">
-        <v>-26517</v>
-      </c>
-      <c r="Q27" s="16">
-        <v>-0.05</v>
-      </c>
-      <c r="R27" s="17" t="inlineStr">
-        <is>
-          <t>Aspiradoras de futones</t>
-        </is>
-      </c>
-      <c r="S27" s="18" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="T27" s="15"/>
-      <c r="U27" s="16"/>
-      <c r="V27" s="15"/>
-      <c r="W27" s="15"/>
-      <c r="X27" s="15"/>
-      <c r="Y27" s="19">
-        <v>1</v>
-      </c>
-      <c r="Z27" s="20">
-        <v>25.99</v>
-      </c>
-      <c r="AA27"/>
-      <c r="AB27"/>
-      <c r="AC27" s="2"/>
-      <c r="AD27" s="19">
-        <v>2</v>
-      </c>
-      <c r="AE27" s="15">
-        <v>0</v>
-      </c>
-      <c r="AF27" s="21">
-        <v>1</v>
-      </c>
-      <c r="AG27" s="22">
-        <v>0</v>
-      </c>
-      <c r="AH27" s="20">
-        <v>4.37</v>
-      </c>
-      <c r="AI27" s="16">
-        <v>0.68</v>
-      </c>
-      <c r="AJ27"/>
-      <c r="AK27" s="13" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="AL27" s="19">
-        <v>88</v>
-      </c>
-      <c r="AM27" s="13" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AN27" s="13"/>
-      <c r="AO27" s="13"/>
-      <c r="AP27"/>
-      <c r="AQ27" s="19">
-        <v>7</v>
-      </c>
-      <c r="AR27" s="19">
-        <v>1</v>
-      </c>
-      <c r="AS27" s="14" t="inlineStr">
-        <is>
-          <t>ALLILUYAA</t>
-        </is>
-      </c>
-      <c r="AT27" s="13" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AU27" s="13" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="AV27" s="14" t="inlineStr">
-        <is>
-          <t>bayuquan LiaoNing 115007 CN</t>
-        </is>
-      </c>
-      <c r="AW27" s="13" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A238ODZG8O3E58</t>
-        </is>
-      </c>
-      <c r="AX27" s="13"/>
-      <c r="AY27" s="13"/>
-      <c r="AZ27" s="13"/>
-      <c r="BA27" s="13"/>
-      <c r="BB27" s="13"/>
-      <c r="BC27" s="13"/>
-      <c r="BD27" s="13"/>
-      <c r="BE27" s="13"/>
-      <c r="BF27" s="13"/>
-      <c r="BG27" s="13"/>
-      <c r="BH27" s="14"/>
-      <c r="BI27" s="23"/>
-      <c r="BJ27" s="23"/>
-      <c r="BK27" s="23"/>
-      <c r="BL27" s="23" t="inlineStr">
-        <is>
-          <t>1 x 1 x 1 cm</t>
-        </is>
-      </c>
-      <c r="BM27" s="23" t="inlineStr">
-        <is>
-          <t>1.00 x 1.00 x 1.00 cm</t>
-        </is>
-      </c>
-      <c r="BN27" s="23" t="inlineStr">
-        <is>
-          <t>430 g</t>
-        </is>
-      </c>
-      <c r="BO27" s="23" t="inlineStr">
-        <is>
-          <t>430.00 g</t>
-        </is>
-      </c>
-      <c r="BP27" s="23" t="inlineStr">
-        <is>
-          <t>25.1 x 20.5 x 11.2 cm</t>
-        </is>
-      </c>
-      <c r="BQ27" s="23" t="inlineStr">
-        <is>
-          <t>25.10 x 20.50 x 11.20 cm</t>
-        </is>
-      </c>
-      <c r="BR27" s="13" t="inlineStr">
         <is>
           <t>小包裹</t>
         </is>
@@ -10312,77 +10060,69 @@
     <hyperlink ref="L19" r:id="rId139" tooltip="https://www.amazon.es/dp/B0FBGQY9YP"/>
     <hyperlink ref="M19" r:id="rId140" tooltip="https://www.amazon.es/b?node=13713592031"/>
     <hyperlink ref="AW19" r:id="rId141" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A3MSJ66TMU8M67"/>
-    <hyperlink ref="C20" r:id="rId142" tooltip="https://www.amazon.es/dp/B0FBX24WH6"/>
-    <hyperlink ref="G20" r:id="rId143" tooltip="https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=syayw"/>
-    <hyperlink ref="J20" r:id="rId144" tooltip="https://www.amazon.es/dp/B0FBX24WH6?psc=1"/>
-    <hyperlink ref="K20" r:id="rId145" tooltip="https://images-na.ssl-images-amazon.com/images/I/61LvanTuKlL._AC_US600_.jpg"/>
-    <hyperlink ref="L20" r:id="rId146" tooltip="https://www.amazon.es/dp/B0FBX24WH6"/>
-    <hyperlink ref="M20" r:id="rId147" tooltip="https://www.amazon.es/b?node=2404713031"/>
+    <hyperlink ref="C20" r:id="rId142" tooltip="https://www.amazon.es/dp/B0FDWVV95V"/>
+    <hyperlink ref="G20" r:id="rId143" tooltip="https://www.amazon.es/stores/JIGOO-ES/page/23E9C8F3-B11D-41BE-B25B-391D7999E178?lp_asin=B0FDWVV95V&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto"/>
+    <hyperlink ref="J20" r:id="rId144" tooltip="https://www.amazon.es/dp/B0FDWVV95V?psc=1"/>
+    <hyperlink ref="K20" r:id="rId145" tooltip="https://images-na.ssl-images-amazon.com/images/I/61tL+-AcL6L._AC_US600_.jpg"/>
+    <hyperlink ref="L20" r:id="rId146" tooltip="https://www.amazon.es/dp/B0FDWVV95V"/>
+    <hyperlink ref="M20" r:id="rId147" tooltip="https://www.amazon.es/b?node=13713592031"/>
     <hyperlink ref="N20" r:id="rId148"/>
-    <hyperlink ref="AW20" r:id="rId149" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A3T9BSXCSWI46M"/>
-    <hyperlink ref="C21" r:id="rId150" tooltip="https://www.amazon.es/dp/B0FDWVV95V"/>
-    <hyperlink ref="G21" r:id="rId151" tooltip="https://www.amazon.es/stores/JIGOO-ES/page/23E9C8F3-B11D-41BE-B25B-391D7999E178?lp_asin=B0FDWVV95V&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto"/>
-    <hyperlink ref="J21" r:id="rId152" tooltip="https://www.amazon.es/dp/B0FDWVV95V?psc=1"/>
-    <hyperlink ref="K21" r:id="rId153" tooltip="https://images-na.ssl-images-amazon.com/images/I/61tL+-AcL6L._AC_US600_.jpg"/>
-    <hyperlink ref="L21" r:id="rId154" tooltip="https://www.amazon.es/dp/B0FDWVV95V"/>
+    <hyperlink ref="AW20" r:id="rId149" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A1LBASE3VLPMEX"/>
+    <hyperlink ref="C21" r:id="rId150" tooltip="https://www.amazon.es/dp/B0FKRC3KQY"/>
+    <hyperlink ref="G21" r:id="rId151" tooltip="https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Yaasier"/>
+    <hyperlink ref="J21" r:id="rId152" tooltip="https://www.amazon.es/dp/B0FKRC3KQY?psc=1"/>
+    <hyperlink ref="K21" r:id="rId153" tooltip="https://images-na.ssl-images-amazon.com/images/I/511XZVAimmL._AC_US600_.jpg"/>
+    <hyperlink ref="L21" r:id="rId154" tooltip="https://www.amazon.es/dp/B0FKRC3KQY"/>
     <hyperlink ref="M21" r:id="rId155" tooltip="https://www.amazon.es/b?node=13713592031"/>
     <hyperlink ref="N21" r:id="rId156"/>
-    <hyperlink ref="AW21" r:id="rId157" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A1LBASE3VLPMEX"/>
-    <hyperlink ref="C22" r:id="rId158" tooltip="https://www.amazon.es/dp/B0FKRC3KQY"/>
-    <hyperlink ref="G22" r:id="rId159" tooltip="https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Yaasier"/>
-    <hyperlink ref="J22" r:id="rId160" tooltip="https://www.amazon.es/dp/B0FKRC3KQY?psc=1"/>
-    <hyperlink ref="K22" r:id="rId161" tooltip="https://images-na.ssl-images-amazon.com/images/I/511XZVAimmL._AC_US600_.jpg"/>
-    <hyperlink ref="L22" r:id="rId162" tooltip="https://www.amazon.es/dp/B0FKRC3KQY"/>
+    <hyperlink ref="AW21" r:id="rId157" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=ATK258MBI08TX"/>
+    <hyperlink ref="C22" r:id="rId158" tooltip="https://www.amazon.es/dp/B0FN3GPQZM"/>
+    <hyperlink ref="G22" r:id="rId159" tooltip="https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Teant"/>
+    <hyperlink ref="J22" r:id="rId160" tooltip="https://www.amazon.es/dp/B0FN3GPQZM?psc=1"/>
+    <hyperlink ref="K22" r:id="rId161" tooltip="https://images-na.ssl-images-amazon.com/images/I/71gt+j80L3L._AC_US600_.jpg"/>
+    <hyperlink ref="L22" r:id="rId162" tooltip="https://www.amazon.es/dp/B0FN3GPQZM"/>
     <hyperlink ref="M22" r:id="rId163" tooltip="https://www.amazon.es/b?node=13713592031"/>
     <hyperlink ref="N22" r:id="rId164"/>
-    <hyperlink ref="AW22" r:id="rId165" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=ATK258MBI08TX"/>
-    <hyperlink ref="C23" r:id="rId166" tooltip="https://www.amazon.es/dp/B0FN3GPQZM"/>
-    <hyperlink ref="G23" r:id="rId167" tooltip="https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Teant"/>
-    <hyperlink ref="J23" r:id="rId168" tooltip="https://www.amazon.es/dp/B0FN3GPQZM?psc=1"/>
-    <hyperlink ref="K23" r:id="rId169" tooltip="https://images-na.ssl-images-amazon.com/images/I/71gt+j80L3L._AC_US600_.jpg"/>
-    <hyperlink ref="L23" r:id="rId170" tooltip="https://www.amazon.es/dp/B0FN3GPQZM"/>
+    <hyperlink ref="AW22" r:id="rId165" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A3EVTWEH1TBVG5"/>
+    <hyperlink ref="C23" r:id="rId166" tooltip="https://www.amazon.es/dp/B0FVS559GZ"/>
+    <hyperlink ref="G23" r:id="rId167" tooltip="https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Yaasier"/>
+    <hyperlink ref="J23" r:id="rId168" tooltip="https://www.amazon.es/dp/B0FVS559GZ?psc=1"/>
+    <hyperlink ref="K23" r:id="rId169" tooltip="https://images-na.ssl-images-amazon.com/images/I/51dJLeDXofL._AC_US600_.jpg"/>
+    <hyperlink ref="L23" r:id="rId170" tooltip="https://www.amazon.es/dp/B0FVS559GZ"/>
     <hyperlink ref="M23" r:id="rId171" tooltip="https://www.amazon.es/b?node=13713592031"/>
     <hyperlink ref="N23" r:id="rId172"/>
-    <hyperlink ref="AW23" r:id="rId173" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A3EVTWEH1TBVG5"/>
-    <hyperlink ref="C24" r:id="rId174" tooltip="https://www.amazon.es/dp/B0FVS559GZ"/>
+    <hyperlink ref="AW23" r:id="rId173" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=ATK258MBI08TX"/>
+    <hyperlink ref="C24" r:id="rId174" tooltip="https://www.amazon.es/dp/B0FYM1D13D"/>
     <hyperlink ref="G24" r:id="rId175" tooltip="https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Yaasier"/>
-    <hyperlink ref="J24" r:id="rId176" tooltip="https://www.amazon.es/dp/B0FVS559GZ?psc=1"/>
+    <hyperlink ref="J24" r:id="rId176" tooltip="https://www.amazon.es/dp/B0FYM1D13D?psc=1"/>
     <hyperlink ref="K24" r:id="rId177" tooltip="https://images-na.ssl-images-amazon.com/images/I/51dJLeDXofL._AC_US600_.jpg"/>
-    <hyperlink ref="L24" r:id="rId178" tooltip="https://www.amazon.es/dp/B0FVS559GZ"/>
+    <hyperlink ref="L24" r:id="rId178" tooltip="https://www.amazon.es/dp/B0FYM1D13D"/>
     <hyperlink ref="M24" r:id="rId179" tooltip="https://www.amazon.es/b?node=13713592031"/>
     <hyperlink ref="N24" r:id="rId180"/>
     <hyperlink ref="AW24" r:id="rId181" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=ATK258MBI08TX"/>
-    <hyperlink ref="C25" r:id="rId182" tooltip="https://www.amazon.es/dp/B0FYM1D13D"/>
-    <hyperlink ref="G25" r:id="rId183" tooltip="https://www.amazon.es/s/ref=bl_dp_s_web_0?ie=UTF8&amp;search-alias=aps&amp;field-keywords=Yaasier"/>
-    <hyperlink ref="J25" r:id="rId184" tooltip="https://www.amazon.es/dp/B0FYM1D13D?psc=1"/>
-    <hyperlink ref="K25" r:id="rId185" tooltip="https://images-na.ssl-images-amazon.com/images/I/51dJLeDXofL._AC_US600_.jpg"/>
-    <hyperlink ref="L25" r:id="rId186" tooltip="https://www.amazon.es/dp/B0FYM1D13D"/>
+    <hyperlink ref="C25" r:id="rId182" tooltip="https://www.amazon.es/dp/B0G4RSJQVT"/>
+    <hyperlink ref="G25" r:id="rId183" tooltip="https://www.amazon.es/stores/Lubluelu/page/6949B717-1950-436B-B468-8BFB57AEF209?lp_asin=B0G4RSJQVT&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto&amp;bl_grd_status=override"/>
+    <hyperlink ref="J25" r:id="rId184" tooltip="https://www.amazon.es/dp/B0G4RSJQVT?psc=1"/>
+    <hyperlink ref="K25" r:id="rId185" tooltip="https://images-na.ssl-images-amazon.com/images/I/71mJa10XC6L._AC_US600_.jpg"/>
+    <hyperlink ref="L25" r:id="rId186" tooltip="https://www.amazon.es/dp/B0G4RSJQVT"/>
     <hyperlink ref="M25" r:id="rId187" tooltip="https://www.amazon.es/b?node=13713592031"/>
     <hyperlink ref="N25" r:id="rId188"/>
-    <hyperlink ref="AW25" r:id="rId189" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=ATK258MBI08TX"/>
-    <hyperlink ref="C26" r:id="rId190" tooltip="https://www.amazon.es/dp/B0G4RSJQVT"/>
-    <hyperlink ref="G26" r:id="rId191" tooltip="https://www.amazon.es/stores/Lubluelu/page/6949B717-1950-436B-B468-8BFB57AEF209?lp_asin=B0G4RSJQVT&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto&amp;bl_grd_status=override"/>
-    <hyperlink ref="J26" r:id="rId192" tooltip="https://www.amazon.es/dp/B0G4RSJQVT?psc=1"/>
-    <hyperlink ref="K26" r:id="rId193" tooltip="https://images-na.ssl-images-amazon.com/images/I/71mJa10XC6L._AC_US600_.jpg"/>
-    <hyperlink ref="L26" r:id="rId194" tooltip="https://www.amazon.es/dp/B0G4RSJQVT"/>
-    <hyperlink ref="M26" r:id="rId195" tooltip="https://www.amazon.es/b?node=13713592031"/>
-    <hyperlink ref="N26" r:id="rId196"/>
-    <hyperlink ref="C27" r:id="rId197" tooltip="https://www.amazon.es/dp/B0GYS43G8G"/>
-    <hyperlink ref="G27" r:id="rId198" tooltip="https://www.amazon.es/stores/ALILILUYAA/page/6F2D9C3F-3247-41D0-93BE-BD3270082609?lp_asin=B0GYS43G8G&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto&amp;bl_grd_status=override"/>
-    <hyperlink ref="J27" r:id="rId199" tooltip="https://www.amazon.es/dp/B0GYS43G8G?psc=1"/>
-    <hyperlink ref="K27" r:id="rId200" tooltip="https://images-na.ssl-images-amazon.com/images/I/51JXrvAAoZL._AC_US600_.jpg"/>
-    <hyperlink ref="L27" r:id="rId201" tooltip="https://www.amazon.es/dp/B0GYS43G8G"/>
-    <hyperlink ref="M27" r:id="rId202" tooltip="https://www.amazon.es/b?node=13713592031"/>
-    <hyperlink ref="N27" r:id="rId203"/>
-    <hyperlink ref="AW27" r:id="rId204" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A238ODZG8O3E58"/>
+    <hyperlink ref="C26" r:id="rId189" tooltip="https://www.amazon.es/dp/B0GYS43G8G"/>
+    <hyperlink ref="G26" r:id="rId190" tooltip="https://www.amazon.es/stores/ALILILUYAA/page/6F2D9C3F-3247-41D0-93BE-BD3270082609?lp_asin=B0GYS43G8G&amp;ref_=ast_bln&amp;store_ref=bl_ast_dp_brandlogo_sto&amp;bl_grd_status=override"/>
+    <hyperlink ref="J26" r:id="rId191" tooltip="https://www.amazon.es/dp/B0GYS43G8G?psc=1"/>
+    <hyperlink ref="K26" r:id="rId192" tooltip="https://images-na.ssl-images-amazon.com/images/I/51JXrvAAoZL._AC_US600_.jpg"/>
+    <hyperlink ref="L26" r:id="rId193" tooltip="https://www.amazon.es/dp/B0GYS43G8G"/>
+    <hyperlink ref="M26" r:id="rId194" tooltip="https://www.amazon.es/b?node=13713592031"/>
+    <hyperlink ref="N26" r:id="rId195"/>
+    <hyperlink ref="AW26" r:id="rId196" tooltip="https://www.amazon.es/gp/help/seller/at-a-glance.html/ref=dp_merchant_link?seller=A238ODZG8O3E58"/>
   </hyperlinks>
-  <drawing r:id="rId205"/>
+  <drawing r:id="rId197"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" style="1" customWidth="1"/>
@@ -10763,25 +10503,6 @@
         <v>0.0</v>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>syayw</t>
-        </is>
-      </c>
-      <c r="B19" s="15">
-        <v>0</v>
-      </c>
-      <c r="C19" s="15">
-        <v>0</v>
-      </c>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="22">
-        <v>0.0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -10790,7 +10511,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" style="1" customWidth="1"/>
@@ -11216,7 +10937,7 @@
     <row r="21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>nousaeg</t>
+          <t>tengjidainzi</t>
         </is>
       </c>
       <c r="B21" s="15">
@@ -11229,25 +10950,6 @@
       <c r="E21" s="15"/>
       <c r="F21" s="20"/>
       <c r="G21" s="22">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>tengjidainzi</t>
-        </is>
-      </c>
-      <c r="B22" s="15">
-        <v>0</v>
-      </c>
-      <c r="C22" s="15">
-        <v>0</v>
-      </c>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="22">
         <v>0.0</v>
       </c>
     </row>

</xml_diff>